<commit_message>
Fix: eliminar imágenes de plantilla que causaban error anchors en ExcelJS
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/template_110.xlsx
+++ b/docs/template_110.xlsx
@@ -22575,273 +22575,6 @@
 </comments>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor>
-    <from>
-      <col>11</col>
-      <colOff>25406</colOff>
-      <row>1</row>
-      <rowOff>8732</rowOff>
-    </from>
-    <to>
-      <col>13</col>
-      <colOff>79585</colOff>
-      <row>2</row>
-      <rowOff>401690</rowOff>
-    </to>
-    <grpSp>
-      <nvGrpSpPr>
-        <cNvPr id="2" name="Grupo 1">
-          <a:hlinkClick xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </cNvPr>
-        <cNvGrpSpPr/>
-      </nvGrpSpPr>
-      <grpSpPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0">
-          <a:off x="8809177" y="51605"/>
-          <a:ext cx="1737666" cy="571598"/>
-          <a:chOff x="7533249" y="626012"/>
-          <a:chExt cx="1687291" cy="571954"/>
-        </a:xfrm>
-      </grpSpPr>
-      <pic>
-        <nvPicPr>
-          <cNvPr id="4" name="Imagen 3"/>
-          <cNvPicPr>
-            <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-          </cNvPicPr>
-        </nvPicPr>
-        <blipFill>
-          <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-          <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:fillRect/>
-          </a:stretch>
-        </blipFill>
-        <spPr>
-          <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:off x="7576514" y="659656"/>
-            <a:ext cx="485946" cy="529056"/>
-          </a:xfrm>
-          <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-            <avLst/>
-          </a:prstGeom>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:prstDash val="solid"/>
-          </a:ln>
-        </spPr>
-      </pic>
-    </grpSp>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="absolute">
-    <from>
-      <col>12</col>
-      <colOff>555334</colOff>
-      <row>1</row>
-      <rowOff>16128</rowOff>
-    </from>
-    <to>
-      <col>17</col>
-      <colOff>398032</colOff>
-      <row>2</row>
-      <rowOff>399830</rowOff>
-    </to>
-    <grpSp>
-      <nvGrpSpPr>
-        <cNvPr id="7" name="Grupo 6">
-          <a:hlinkClick xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
-        </cNvPr>
-        <cNvGrpSpPr/>
-      </nvGrpSpPr>
-      <grpSpPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0">
-          <a:off x="10230153" y="60906"/>
-          <a:ext cx="1734834" cy="568057"/>
-          <a:chOff x="6981288" y="3287542"/>
-          <a:chExt cx="1654001" cy="575764"/>
-        </a:xfrm>
-      </grpSpPr>
-      <pic>
-        <nvPicPr>
-          <cNvPr id="10" name="Imagen 9"/>
-          <cNvPicPr>
-            <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-          </cNvPicPr>
-        </nvPicPr>
-        <blipFill>
-          <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
-          <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:fillRect/>
-          </a:stretch>
-        </blipFill>
-        <spPr>
-          <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:off x="7000545" y="3321049"/>
-            <a:ext cx="527101" cy="514747"/>
-          </a:xfrm>
-          <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-            <avLst/>
-          </a:prstGeom>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:prstDash val="solid"/>
-          </a:ln>
-        </spPr>
-      </pic>
-    </grpSp>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>15</col>
-      <colOff>13656</colOff>
-      <row>1</row>
-      <rowOff>122903</rowOff>
-    </from>
-    <to>
-      <col>18</col>
-      <colOff>419251</colOff>
-      <row>2</row>
-      <rowOff>324724</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="11" name="Imagen 10">
-          <a:hlinkClick xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
-        </cNvPr>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="12047541" y="162908"/>
-          <a:ext cx="1223162" cy="380891"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>3</col>
-      <colOff>190500</colOff>
-      <row>0</row>
-      <rowOff>57150</rowOff>
-    </from>
-    <to>
-      <col>3</col>
-      <colOff>1998346</colOff>
-      <row>1</row>
-      <rowOff>365313</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Imagen 1">
-          <a:hlinkClick xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" tooltip="Visitar sitio web" r:id="rId1"/>
-        </cNvPr>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="5000625" y="53340"/>
-          <a:ext cx="1807846" cy="635823"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>190500</colOff>
-      <row>0</row>
-      <rowOff>104140</rowOff>
-    </from>
-    <to>
-      <col>6</col>
-      <colOff>114608</colOff>
-      <row>1</row>
-      <rowOff>301780</rowOff>
-    </to>
-    <grpSp>
-      <nvGrpSpPr>
-        <cNvPr id="3" name="Grupo 2">
-          <a:hlinkClick xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" tooltip="Descargar otras herramientas" r:id="rId3"/>
-        </cNvPr>
-        <cNvGrpSpPr/>
-      </nvGrpSpPr>
-      <grpSpPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0">
-          <a:off x="7171765" y="102235"/>
-          <a:ext cx="1694637" cy="524516"/>
-          <a:chOff x="7162800" y="107950"/>
-          <a:chExt cx="1683058" cy="524030"/>
-        </a:xfrm>
-      </grpSpPr>
-      <pic>
-        <nvPicPr>
-          <cNvPr id="5" name="Imagen 4"/>
-          <cNvPicPr>
-            <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-          </cNvPicPr>
-        </nvPicPr>
-        <blipFill>
-          <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
-          <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:fillRect/>
-          </a:stretch>
-        </blipFill>
-        <spPr>
-          <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:off x="7205956" y="138775"/>
-            <a:ext cx="484727" cy="484727"/>
-          </a:xfrm>
-          <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-            <avLst/>
-          </a:prstGeom>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:prstDash val="solid"/>
-          </a:ln>
-        </spPr>
-      </pic>
-    </grpSp>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
@@ -26229,7 +25962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T57"/>
+  <dimension ref="A2:T57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="1.33203125" customWidth="1" style="1506" min="1" max="1"/>
@@ -26240,7 +25973,7 @@
     <col width="13.109375" bestFit="1" customWidth="1" style="1506" min="12" max="12"/>
     <col width="16" bestFit="1" customWidth="1" style="1506" min="14" max="14"/>
     <col hidden="1" width="14.33203125" customWidth="1" style="1506" min="15" max="15"/>
-    <col hidden="1" style="1506" min="16" max="17"/>
+    <col hidden="1" width="13" customWidth="1" style="1506" min="16" max="17"/>
     <col width="17.88671875" bestFit="1" customWidth="1" style="1506" min="19" max="19"/>
     <col width="19" customWidth="1" style="1506" min="20" max="20"/>
   </cols>
@@ -26830,7 +26563,6 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
@@ -26842,7 +26574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.33203125" defaultRowHeight="15.6"/>
   <cols>
     <col width="1.33203125" customWidth="1" style="590" min="1" max="1"/>
@@ -27194,12 +26926,6 @@
       <c r="H32" s="597" t="n"/>
       <c r="I32" s="597" t="n"/>
     </row>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
     <row r="39">
       <c r="B39" s="608" t="n">
         <v>0</v>
@@ -27223,8 +26949,6 @@
     <row r="43">
       <c r="B43" s="608" t="n"/>
     </row>
-    <row r="44"/>
-    <row r="45"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" algorithmName="SHA-512" sheet="1" objects="1" insertRows="1" insertHyperlinks="0" autoFilter="0" scenarios="1" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" saltValue="d8/754m7aeojz5pxqbD7Jg==" formatRows="0" sort="0" spinCount="100000" hashValue="x6C4DFWiHgnnNLk2A93OOFpqn3c3G5kRySEsPovsseJno221alpsJb53RUfMl971RgvyOFx+m19/O7BTlULtZQ=="/>
   <mergeCells count="15">
@@ -27261,6 +26985,5 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix: reconstruir plantilla sin comments/images que rompían ExcelJS
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/template_110.xlsx
+++ b/docs/template_110.xlsx
@@ -22533,48 +22533,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Autor</author>
-  </authors>
-  <commentList>
-    <comment ref="G19" authorId="0" shapeId="0">
-      <text>
-        <t>Consulte los códigos de la actividades económicas, en la cartilla de instrucciones o en la pág. www.dian.gov.co/servicios/formularios</t>
-      </text>
-    </comment>
-    <comment ref="E60" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">01. Declarante                        05. Agente oficioso       09. Curador          13. Liquidador
-02. Representante legal          06. Padres                    10. Donatario        14. Mandatario
-03. Administrador privado      07. Tutor                     11. Heredero         15. Funcionario autorizado
-04. Apoderado                        08. Albacea                   12. Asignatario </t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>tc={69AFA52E-0314-480B-ABF3-4F5456EBDD0B}</author>
-  </authors>
-  <commentList>
-    <comment ref="D19" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">[Comentario encadenado]
-Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
-Comentario:
-    Ingresos Economía naranja exentos
-https://www.youtube.com/watch?v=vzz7c1dVX9Q </t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
@@ -22963,7 +22921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM69"/>
+  <dimension ref="A1:AN69"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="5.33203125" customWidth="1" style="1506" min="1" max="5"/>
@@ -25951,7 +25909,6 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="119" horizontalDpi="1200" verticalDpi="1200"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -25962,7 +25919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:T57"/>
+  <dimension ref="A1:AN57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="1.33203125" customWidth="1" style="1506" min="1" max="1"/>
@@ -25973,7 +25930,7 @@
     <col width="13.109375" bestFit="1" customWidth="1" style="1506" min="12" max="12"/>
     <col width="16" bestFit="1" customWidth="1" style="1506" min="14" max="14"/>
     <col hidden="1" width="14.33203125" customWidth="1" style="1506" min="15" max="15"/>
-    <col hidden="1" width="13" customWidth="1" style="1506" min="16" max="17"/>
+    <col hidden="1" style="1506" min="16" max="17"/>
     <col width="17.88671875" bestFit="1" customWidth="1" style="1506" min="19" max="19"/>
     <col width="19" customWidth="1" style="1506" min="20" max="20"/>
   </cols>
@@ -26563,7 +26520,6 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -26574,7 +26530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:AN43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.33203125" defaultRowHeight="15.6"/>
   <cols>
     <col width="1.33203125" customWidth="1" style="590" min="1" max="1"/>
@@ -26926,6 +26882,12 @@
       <c r="H32" s="597" t="n"/>
       <c r="I32" s="597" t="n"/>
     </row>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
     <row r="39">
       <c r="B39" s="608" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Fix: eliminar externalLinks de plantilla (causa error anchors) + botón X para borrar balance
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/template_110.xlsx
+++ b/docs/template_110.xlsx
@@ -10,9 +10,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impuesto mínimo" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ANT" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <externalReferences>
-    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
-  </externalReferences>
   <definedNames>
     <definedName name="\0">#REF!</definedName>
     <definedName name="\a">#REF!</definedName>
@@ -22533,102 +22530,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="ESTADO DE RESULTADOS"/>
-      <sheetName val="Libro mayor 2025"/>
-      <sheetName val="Libro mayor 21"/>
-      <sheetName val="PYG 2020-2019"/>
-      <sheetName val="Libro mayor 2024"/>
-      <sheetName val="EEFF"/>
-      <sheetName val="Worksheet ind y c bogotá"/>
-      <sheetName val="Notas"/>
-      <sheetName val="FLE"/>
-      <sheetName val="ECP"/>
-      <sheetName val="Renta"/>
-      <sheetName val="ICA"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1">
-        <row r="8">
-          <cell r="J8">
-            <v>679795269.19000006</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="H25">
-            <v>20109703.260000002</v>
-          </cell>
-        </row>
-        <row r="28">
-          <cell r="H28">
-            <v>4188796721.25</v>
-          </cell>
-        </row>
-        <row r="60">
-          <cell r="J60">
-            <v>201894352</v>
-          </cell>
-        </row>
-        <row r="68">
-          <cell r="I68">
-            <v>32178</v>
-          </cell>
-        </row>
-        <row r="70">
-          <cell r="I70">
-            <v>67438987.609999999</v>
-          </cell>
-        </row>
-        <row r="73">
-          <cell r="I73">
-            <v>73230.09</v>
-          </cell>
-        </row>
-        <row r="74">
-          <cell r="H74">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="77">
-          <cell r="I77">
-            <v>23681483</v>
-          </cell>
-        </row>
-        <row r="79">
-          <cell r="I79">
-            <v>274777945.83999997</v>
-          </cell>
-        </row>
-        <row r="92">
-          <cell r="I92">
-            <v>109041646.33</v>
-          </cell>
-        </row>
-        <row r="101">
-          <cell r="I101">
-            <v>0</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>

</xml_diff>

<commit_message>
Quitar Impuesto Mínimo, nuevo Anticipo diseño ExogenaDIAN
- Eliminada hoja Impuesto Mínimo de la plantilla y del código
- Plantilla solo tiene hoja 110 (formato DIAN limpio)
- Nueva hoja Anticipo de Renta con diseño propio:
  3 opciones (75%, promedio, 25%), datos base, resultado con fórmulas
- Colores y tipografía ExogenaDIAN (azul navy, verde, gris)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/template_110.xlsx
+++ b/docs/template_110.xlsx
@@ -7,8 +7,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="110" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impuesto mínimo" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ANT" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -10501,7 +10499,7 @@
         <v>95</v>
       </c>
       <c r="AC38" s="926">
-        <f>'Impuesto mínimo'!E34</f>
+        <v>0</v>
         <v/>
       </c>
       <c r="AD38" s="1553" t="n"/>
@@ -12089,1042 +12087,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="119" horizontalDpi="1200" verticalDpi="1200"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="FFFFC000"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AN57"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="1.33203125" customWidth="1" style="1506" min="1" max="1"/>
-    <col width="12.6640625" customWidth="1" style="1506" min="2" max="2"/>
-    <col width="1.109375" customWidth="1" style="1506" min="3" max="3"/>
-    <col width="29" customWidth="1" style="1506" min="4" max="4"/>
-    <col width="15.109375" customWidth="1" style="1506" min="5" max="5"/>
-    <col width="13.109375" bestFit="1" customWidth="1" style="1506" min="12" max="12"/>
-    <col width="16" bestFit="1" customWidth="1" style="1506" min="14" max="14"/>
-    <col hidden="1" width="14.33203125" customWidth="1" style="1506" min="15" max="15"/>
-    <col hidden="1" style="1506" min="16" max="17"/>
-    <col width="17.88671875" bestFit="1" customWidth="1" style="1506" min="19" max="19"/>
-    <col width="19" customWidth="1" style="1506" min="20" max="20"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="3.45" customFormat="1" customHeight="1" s="486"/>
-    <row r="2" customFormat="1" s="486">
-      <c r="B2" s="487" t="inlineStr">
-        <is>
-          <t>TASA  MÍNIMA DE TRIBUTACIÓN EN RENTA (Parágrafo 6 art. 240 ET ) REFORMA TRIBUTARIA 2022</t>
-        </is>
-      </c>
-      <c r="C2" s="488" t="n"/>
-      <c r="D2" s="488" t="n"/>
-      <c r="E2" s="488" t="n"/>
-      <c r="F2" s="488" t="n"/>
-      <c r="G2" s="488" t="n"/>
-      <c r="H2" s="488" t="n"/>
-      <c r="I2" s="488" t="n"/>
-      <c r="J2" s="488" t="n"/>
-      <c r="K2" s="488" t="n"/>
-    </row>
-    <row r="3" ht="34.2" customFormat="1" customHeight="1" s="486">
-      <c r="B3" s="1009" t="inlineStr">
-        <is>
-          <t>Esta tasa mínima se denominará Tasa de Tributación Depurada (TTD) la cual no podrá ser inferior al 15% y será el resultado de dividir el Impuesto Depurado (ID) sobre la Utilidad Depurada (UD), así:</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="7.95" customFormat="1" customHeight="1" s="486"/>
-    <row r="5" customFormat="1" s="486">
-      <c r="B5" s="1012" t="inlineStr">
-        <is>
-          <t>𝑇𝑇𝐷= 𝐼𝐷 / 𝑈𝐷</t>
-        </is>
-      </c>
-      <c r="C5" s="489" t="n"/>
-      <c r="D5" s="489" t="inlineStr">
-        <is>
-          <t>Impuesto Depurado (ID)</t>
-        </is>
-      </c>
-      <c r="E5" s="490" t="inlineStr">
-        <is>
-          <t>𝐼𝐷=𝐼𝑁𝑅+𝐷𝑇𝐶−𝐼𝑅𝑃</t>
-        </is>
-      </c>
-      <c r="F5" s="490" t="n"/>
-      <c r="G5" s="490" t="n"/>
-      <c r="H5" s="490" t="n"/>
-      <c r="K5" s="486" t="inlineStr">
-        <is>
-          <t>Impuesto neto total</t>
-        </is>
-      </c>
-      <c r="M5" s="1579">
-        <f>+E36</f>
-        <v/>
-      </c>
-      <c r="O5" s="1580" t="n"/>
-    </row>
-    <row r="6" customFormat="1" s="486">
-      <c r="C6" s="489" t="n"/>
-      <c r="D6" s="489" t="inlineStr">
-        <is>
-          <t>Utilidad Depurada (UD)</t>
-        </is>
-      </c>
-      <c r="E6" s="489" t="inlineStr">
-        <is>
-          <t>𝑈𝐷=𝑈𝐶+𝐷𝑃𝐴𝑅𝐿−𝐼𝑁𝐶𝑅𝑁𝐺𝑂−𝑉𝐼𝑀𝑃𝑃−𝑉𝑁𝐺𝑂−𝑅𝐸−𝐶</t>
-        </is>
-      </c>
-      <c r="F6" s="489" t="n"/>
-      <c r="G6" s="489" t="n"/>
-      <c r="H6" s="489" t="n"/>
-      <c r="M6" s="492" t="inlineStr"/>
-      <c r="N6" s="493" t="n"/>
-      <c r="O6" s="1580" t="n"/>
-    </row>
-    <row r="7" ht="9" customFormat="1" customHeight="1" s="486"/>
-    <row r="8" ht="22.5" customFormat="1" customHeight="1" s="486">
-      <c r="B8" s="494" t="inlineStr">
-        <is>
-          <t>Digite información para hacer simulación del efecto</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="9" customFormat="1" customHeight="1" s="486"/>
-    <row r="10" customFormat="1" s="486">
-      <c r="B10" s="1015" t="inlineStr">
-        <is>
-          <t>Digitar información</t>
-        </is>
-      </c>
-      <c r="D10" s="1581" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="486" t="inlineStr">
-        <is>
-          <t>INR: Impuesto neto de renta.</t>
-        </is>
-      </c>
-      <c r="H10" s="496" t="inlineStr">
-        <is>
-          <t>(Despues de desc.. Tributarios)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" customFormat="1" s="486">
-      <c r="B11" s="1214" t="n"/>
-      <c r="D11" s="1581" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="486" t="inlineStr">
-        <is>
-          <t>DTC: Descuentos tributarios o créditos tributarios por aplicación de tratados para evitar la doble imposición y el establecido en el artículo 254 del Estatuto Tributario.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" customFormat="1" s="486">
-      <c r="B12" s="1214" t="n"/>
-      <c r="D12" s="1581" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="486" t="inlineStr">
-        <is>
-          <t>IRP: Impuesto sobre la renta por rentas pasivas provenientes de entidades controladas del exterior. Se calculará multiplicando la renta líquida pasiva por la tarifa general del artículo 240 del Estatuto Tributario (renta líquida pasiva x tarifa general).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" customFormat="1" s="486">
-      <c r="B13" s="1214" t="n"/>
-      <c r="D13" s="1580" t="n"/>
-    </row>
-    <row r="14" customFormat="1" s="486">
-      <c r="B14" s="1214" t="n"/>
-      <c r="D14" s="1581" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="486" t="inlineStr">
-        <is>
-          <t>UC: Utilidad contable o financiera antes de impuestos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" customFormat="1" s="486">
-      <c r="B15" s="1214" t="n"/>
-      <c r="D15" s="1581" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="486" t="inlineStr">
-        <is>
-          <t>DPARL: Diferencias permanentes consagradas en la ley y que aumentan la renta líquida.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" customFormat="1" s="486">
-      <c r="B16" s="1214" t="n"/>
-      <c r="D16" s="1581" t="n"/>
-      <c r="E16" s="486" t="inlineStr">
-        <is>
-          <t>INCRNGO: Ingresos no constitutivos de renta ni ganancia ocasional, que afectan la utilidad contable o financiera.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" customFormat="1" s="486">
-      <c r="B17" s="1214" t="n"/>
-      <c r="D17" s="1581" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="486" t="inlineStr">
-        <is>
-          <t>VIMPP: Valor ingreso método de participación patrimonial del respectivo año gravable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" customFormat="1" s="486">
-      <c r="B18" s="1214" t="n"/>
-      <c r="D18" s="1581" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="486" t="inlineStr">
-        <is>
-          <t>VNGO: Valor neto de ingresos por ganancia ocasional que afectan la utilidad contable o financiera.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customFormat="1" customHeight="1" s="486">
-      <c r="B19" s="1214" t="n"/>
-      <c r="D19" s="1581" t="n"/>
-      <c r="E19" s="486" t="inlineStr">
-        <is>
-          <t>RE: Rentas exentas por aplicación de tratados para evitar la doble imposición – CAN, las percibidas por el régimen de compañías holding colombianas -CHC y las rentas exentas de que tratan los literales a) y b) del numeral 4 del artículo 235-2 del Estatuto Tributario.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" customFormat="1" s="486">
-      <c r="B20" s="1229" t="n"/>
-      <c r="D20" s="1581" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="486" t="inlineStr">
-        <is>
-          <t>C: Compensación de pérdidas fiscales o excesos de renta presuntiva tomados en el año gravable y que no afectaron la utilidad contable del periodo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" customFormat="1" s="486"/>
-    <row r="22" customFormat="1" s="486">
-      <c r="A22" s="497" t="n"/>
-      <c r="B22" s="498" t="n"/>
-      <c r="C22" s="498" t="n"/>
-      <c r="D22" s="1582" t="inlineStr">
-        <is>
-          <t>TTD</t>
-        </is>
-      </c>
-      <c r="E22" s="1583">
-        <f>+D10+D11-D12</f>
-        <v/>
-      </c>
-      <c r="F22" s="1584">
-        <f>IFERROR(+E22/E23,0)</f>
-        <v/>
-      </c>
-      <c r="G22" s="498" t="n"/>
-      <c r="H22" s="498" t="n"/>
-      <c r="I22" s="498" t="n"/>
-      <c r="J22" s="498" t="n"/>
-      <c r="K22" s="500" t="n"/>
-    </row>
-    <row r="23" customFormat="1" s="486">
-      <c r="A23" s="501" t="n"/>
-      <c r="B23" s="502" t="n"/>
-      <c r="C23" s="502" t="n"/>
-      <c r="D23" s="1537" t="n"/>
-      <c r="E23" s="1585">
-        <f>+D14+D15-D16-D17-D18-D19-D20</f>
-        <v/>
-      </c>
-      <c r="F23" s="1537" t="n"/>
-      <c r="G23" s="502" t="n"/>
-      <c r="H23" s="502" t="n"/>
-      <c r="I23" s="502" t="n"/>
-      <c r="J23" s="502" t="n"/>
-      <c r="K23" s="504" t="n"/>
-    </row>
-    <row r="24" customFormat="1" s="486"/>
-    <row r="25" customFormat="1" s="486">
-      <c r="B25" s="494" t="inlineStr">
-        <is>
-          <t>Cuando la Tasa de Tributación Depurada (TTD) sea inferior al 15%, se deberá determinar el valor del Impuesto a Adicionar (IA) para alcanzar la tasa del 15%, así:</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" customFormat="1" s="486"/>
-    <row r="27" customFormat="1" s="486">
-      <c r="B27" s="1009" t="inlineStr">
-        <is>
-          <t>1. Para los contribuyentes sujetos a este artículo y al artículo 240-1 del Estatuto Tributario, cuyos estados financieros no sean objeto de consolidación, la diferencia positiva entre la Utilidad Depurada (UD) multiplicada por el 15% y el Impuesto Depurado (ID), será un mayor valor del impuesto sobre la renta, que deberá adicionarse al impuesto sobre la renta (IA).</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" customFormat="1" s="486"/>
-    <row r="29" customFormat="1" s="486"/>
-    <row r="30" customFormat="1" s="486"/>
-    <row r="31" customFormat="1" s="486">
-      <c r="B31" s="489" t="inlineStr">
-        <is>
-          <t>𝐼𝐴=(𝑈𝐷∗15%)−𝐼𝐷</t>
-        </is>
-      </c>
-      <c r="C31" s="489" t="n"/>
-      <c r="D31" s="489" t="n"/>
-      <c r="E31" s="489" t="n"/>
-      <c r="F31" s="489" t="n"/>
-      <c r="G31" s="489" t="n"/>
-      <c r="H31" s="489" t="n"/>
-    </row>
-    <row r="32" customFormat="1" s="486"/>
-    <row r="33" customFormat="1" s="486">
-      <c r="B33" s="505" t="n"/>
-      <c r="C33" s="506" t="n"/>
-      <c r="D33" s="506" t="n"/>
-      <c r="E33" s="506" t="n"/>
-      <c r="F33" s="506" t="n"/>
-      <c r="G33" s="506" t="n"/>
-      <c r="H33" s="506" t="n"/>
-      <c r="I33" s="506" t="n"/>
-      <c r="J33" s="506" t="n"/>
-      <c r="K33" s="507" t="n"/>
-    </row>
-    <row r="34" customFormat="1" s="486">
-      <c r="B34" s="508" t="inlineStr">
-        <is>
-          <t>Impuesto a adicionar IA:</t>
-        </is>
-      </c>
-      <c r="C34" s="509" t="n"/>
-      <c r="D34" s="509" t="n"/>
-      <c r="E34" s="1586">
-        <f>IF(F22&lt;15%,((E23*15%)-E22),0)</f>
-        <v/>
-      </c>
-      <c r="F34" s="509" t="n"/>
-      <c r="K34" s="511" t="n"/>
-      <c r="L34" s="1587">
-        <f>+E34-E22</f>
-        <v/>
-      </c>
-      <c r="N34" s="1588">
-        <f>+D14*15%</f>
-        <v/>
-      </c>
-      <c r="P34" s="1587" t="n"/>
-    </row>
-    <row r="35" customFormat="1" s="486">
-      <c r="B35" s="512" t="n"/>
-      <c r="K35" s="511" t="n"/>
-      <c r="N35" s="1588">
-        <f>ROUND(+E23*15%,0)</f>
-        <v/>
-      </c>
-      <c r="S35" s="1589" t="n"/>
-      <c r="T35" s="1590" t="n"/>
-    </row>
-    <row r="36" customFormat="1" s="486">
-      <c r="B36" s="513" t="inlineStr">
-        <is>
-          <t>TOTAL IMPUESTO NETO</t>
-        </is>
-      </c>
-      <c r="C36" s="514" t="n"/>
-      <c r="D36" s="514" t="n"/>
-      <c r="E36" s="1591">
-        <f>+D10+E34</f>
-        <v/>
-      </c>
-      <c r="F36" s="514" t="n"/>
-      <c r="G36" s="516">
-        <f>IF(E34&lt;1,"No hay adición de impuesto","")</f>
-        <v/>
-      </c>
-      <c r="K36" s="511" t="n"/>
-    </row>
-    <row r="37" customFormat="1" s="486">
-      <c r="B37" s="517" t="n"/>
-      <c r="C37" s="518" t="n"/>
-      <c r="D37" s="518" t="n"/>
-      <c r="E37" s="518" t="n"/>
-      <c r="F37" s="518" t="n"/>
-      <c r="G37" s="518" t="n"/>
-      <c r="H37" s="518" t="n"/>
-      <c r="I37" s="518" t="n"/>
-      <c r="J37" s="518" t="n"/>
-      <c r="K37" s="519" t="n"/>
-      <c r="N37" s="1592">
-        <f>ROUND(E34,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" customFormat="1" s="486"/>
-    <row r="39" customFormat="1" s="521">
-      <c r="B39" s="520" t="inlineStr">
-        <is>
-          <t>Desde punto hacia abajo no se ha formulado</t>
-        </is>
-      </c>
-      <c r="M39" s="520" t="n"/>
-    </row>
-    <row r="40" customFormat="1" s="486">
-      <c r="B40" s="522" t="n"/>
-      <c r="M40" s="522" t="n"/>
-    </row>
-    <row r="41" customFormat="1" s="486">
-      <c r="B41" s="522" t="n"/>
-      <c r="M41" s="522" t="n"/>
-    </row>
-    <row r="42" customFormat="1" s="486">
-      <c r="B42" s="1010" t="inlineStr">
-        <is>
-          <t>2. Los contribuyentes residentes fiscales en Colombia cuyos estados financieros sean objeto de consolidación en Colombia, deberán realizar el siguiente procedimiento:
-2.1. Calcular la Tasa de Tributación Depurada del Grupo (TTDG) dividiendo la sumatoria de los Impuestos Depurados (ΣID) de cada contribuyente residente fiscal en Colombia objeto de consolidación por la sumatoria de la Utilidad Depurada (ΣUD) de cada contribuyente residente fiscal en Colombia cuyos estados financieros son objeto de consolidación, así:</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="70.2" customFormat="1" customHeight="1" s="486"/>
-    <row r="44" customFormat="1" s="486">
-      <c r="B44" s="489" t="inlineStr">
-        <is>
-          <t>𝑇𝑇𝐷𝐺= Σ𝐼𝐷 / Σ𝑈𝐷</t>
-        </is>
-      </c>
-      <c r="C44" s="489" t="n"/>
-      <c r="D44" s="489" t="n"/>
-      <c r="E44" s="489" t="n"/>
-      <c r="F44" s="489" t="n"/>
-    </row>
-    <row r="45" customFormat="1" s="486"/>
-    <row r="46" customFormat="1" s="486"/>
-    <row r="47" ht="43.95" customFormat="1" customHeight="1" s="486">
-      <c r="B47" s="1011" t="inlineStr">
-        <is>
-          <t>2.2. Si el resultado es inferior al 15%, se deberá calcular el Impuesto a Adicionar por el Grupo (IAG) a partir de la diferencia entre la sumatoria de la Utilidad Depurada (ΣUD) multiplicada por el 15% menos la sumatoria del Impuesto Depurado (ΣID) de cada contribuyente, cuyos estados financieros se consolidan, así:</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" hidden="1" customFormat="1" s="486"/>
-    <row r="49" customFormat="1" s="486">
-      <c r="B49" s="489" t="inlineStr">
-        <is>
-          <t>𝐼𝐴𝐺=(Σ𝑈𝐷∗15%)−Σ𝐼𝐷</t>
-        </is>
-      </c>
-      <c r="C49" s="489" t="n"/>
-      <c r="D49" s="489" t="n"/>
-      <c r="E49" s="489" t="n"/>
-      <c r="F49" s="489" t="n"/>
-    </row>
-    <row r="50" customFormat="1" s="486"/>
-    <row r="51" customFormat="1" s="486">
-      <c r="B51" s="1009" t="inlineStr">
-        <is>
-          <t>2.3. Para calcular el Impuesto a Adicionar (IA) de cada contribuyente residente fiscal en Colombia, se deberá multiplicar el Impuesto a Adicionar por el Grupo (IAG) por el porcentaje que dé como resultado la división de la Utilidad Depurada) de cada contribuyente con utilidad depurada mayor a cero (UDβ sobre la sumatoria de las Utilidades Depuradas de los contribuyentes con Utilidades Depuradas mayores a cero (ΣUDβ), así:</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="28.2" customFormat="1" customHeight="1" s="486"/>
-    <row r="53" customFormat="1" s="486"/>
-    <row r="54" customFormat="1" s="486">
-      <c r="B54" s="489" t="inlineStr">
-        <is>
-          <t>𝐼𝐴=𝐼𝐴𝐺 × (𝑈𝐷𝛽 / Σ𝑈𝐷𝛽)</t>
-        </is>
-      </c>
-      <c r="C54" s="489" t="n"/>
-      <c r="D54" s="489" t="n"/>
-      <c r="E54" s="489" t="n"/>
-      <c r="F54" s="489" t="n"/>
-    </row>
-    <row r="55" customFormat="1" s="486"/>
-    <row r="56" ht="142.2" customFormat="1" customHeight="1" s="486">
-      <c r="B56" s="1010" t="inlineStr">
-        <is>
-          <t>Lo dispuesto en este parágrafo no aplica para:
-a) Las sociedades que se constituyeron como Zonas Económicas y Sociales Especiales -ZESE durante el periodo que su tarifa del impuesto sobre la renta sea del cero por ciento (0%), las sociedades que aplican el incentivo tributario de las zonas más afectadas por el conflicto armado -ZOMAC, las sociedades de que tratan los parágrafos 5 y 7 del presente artículo, siempre y cuando no estén obligadas a presentar el informe país por país de conformidad con lo establecido en el artículo 260-5 del Estatuto Tributario.
-b) Las sociedades de que trata el parágrafo 1 del presente artículo.
-De igual forma no aplica lo indicado en este parágrafo para aquellos contribuyentes cuyos estados financieros no sean objeto de consolidación y su Utilidad Depurada (UD) sea igual o menor a cero, o para los contribuyentes cuyos estados financieros sean objeto de consolidación y la sumatoria de la Utilidad Depurada (ΣUD) sea igual o menor a cero.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" hidden="1" customFormat="1" s="486"/>
-    <row r="58" customFormat="1" s="486"/>
-    <row r="59" customFormat="1" s="486"/>
-    <row r="60" customFormat="1" s="486"/>
-    <row r="61" customFormat="1" s="486"/>
-    <row r="62" customFormat="1" s="486"/>
-    <row r="63" customFormat="1" s="486"/>
-    <row r="64" customFormat="1" s="486"/>
-    <row r="65" customFormat="1" s="486"/>
-    <row r="66" customFormat="1" s="486"/>
-    <row r="67" customFormat="1" s="486"/>
-    <row r="68" customFormat="1" s="486"/>
-    <row r="69" customFormat="1" s="486"/>
-    <row r="70" customFormat="1" s="486"/>
-    <row r="71" customFormat="1" s="486"/>
-    <row r="72" customFormat="1" s="486"/>
-    <row r="73" customFormat="1" s="486"/>
-    <row r="74" customFormat="1" s="486"/>
-    <row r="75" customFormat="1" s="486"/>
-    <row r="76" customFormat="1" s="486"/>
-    <row r="77" customFormat="1" s="486"/>
-    <row r="78" customFormat="1" s="486"/>
-    <row r="79" customFormat="1" s="486"/>
-    <row r="80" customFormat="1" s="486"/>
-    <row r="81" customFormat="1" s="486"/>
-    <row r="82" customFormat="1" s="486"/>
-    <row r="83" customFormat="1" s="486"/>
-    <row r="84" customFormat="1" s="486"/>
-    <row r="85" customFormat="1" s="486"/>
-    <row r="86" customFormat="1" s="486"/>
-    <row r="87" customFormat="1" s="486"/>
-    <row r="88" customFormat="1" s="486"/>
-    <row r="89" customFormat="1" s="486"/>
-    <row r="90" customFormat="1" s="486"/>
-    <row r="91" customFormat="1" s="486"/>
-    <row r="92" customFormat="1" s="486"/>
-    <row r="93" customFormat="1" s="486"/>
-    <row r="94" customFormat="1" s="486"/>
-    <row r="95" customFormat="1" s="486"/>
-    <row r="96" customFormat="1" s="486"/>
-    <row r="97" customFormat="1" s="486"/>
-    <row r="98" customFormat="1" s="486"/>
-    <row r="99" customFormat="1" s="486"/>
-    <row r="100" customFormat="1" s="486"/>
-    <row r="101" customFormat="1" s="486"/>
-    <row r="102" customFormat="1" s="486"/>
-    <row r="103" customFormat="1" s="486"/>
-    <row r="104" customFormat="1" s="486"/>
-    <row r="105" customFormat="1" s="486"/>
-    <row r="106" customFormat="1" s="486"/>
-    <row r="107" customFormat="1" s="486"/>
-    <row r="108" customFormat="1" s="486"/>
-    <row r="109" customFormat="1" s="486"/>
-    <row r="110" customFormat="1" s="486"/>
-    <row r="111" customFormat="1" s="486"/>
-    <row r="112" customFormat="1" s="486"/>
-    <row r="113" customFormat="1" s="486"/>
-    <row r="114" customFormat="1" s="486"/>
-    <row r="115" customFormat="1" s="486"/>
-    <row r="116" customFormat="1" s="486"/>
-    <row r="117" customFormat="1" s="486"/>
-    <row r="118" customFormat="1" s="486"/>
-    <row r="119" customFormat="1" s="486"/>
-    <row r="120" customFormat="1" s="486"/>
-    <row r="121" customFormat="1" s="486"/>
-    <row r="122" customFormat="1" s="486"/>
-    <row r="123" customFormat="1" s="486"/>
-    <row r="124" customFormat="1" s="486"/>
-    <row r="125" customFormat="1" s="486"/>
-    <row r="126" customFormat="1" s="486"/>
-    <row r="127" customFormat="1" s="486"/>
-    <row r="128" customFormat="1" s="486"/>
-    <row r="129" customFormat="1" s="486"/>
-    <row r="130" customFormat="1" s="486"/>
-    <row r="131" customFormat="1" s="486"/>
-    <row r="132" customFormat="1" s="486"/>
-    <row r="133" customFormat="1" s="486"/>
-    <row r="134" customFormat="1" s="486"/>
-    <row r="135" customFormat="1" s="486"/>
-    <row r="136" customFormat="1" s="486"/>
-    <row r="137" customFormat="1" s="486"/>
-    <row r="138" customFormat="1" s="486"/>
-    <row r="139" customFormat="1" s="486"/>
-    <row r="140" customFormat="1" s="486"/>
-    <row r="141" customFormat="1" s="486"/>
-    <row r="142" customFormat="1" s="486"/>
-    <row r="143" customFormat="1" s="486"/>
-    <row r="144" customFormat="1" s="486"/>
-    <row r="145" customFormat="1" s="486"/>
-    <row r="146" customFormat="1" s="486"/>
-    <row r="147" customFormat="1" s="486"/>
-    <row r="148" customFormat="1" s="486"/>
-    <row r="149" customFormat="1" s="486"/>
-    <row r="150" customFormat="1" s="486"/>
-    <row r="151" customFormat="1" s="486"/>
-    <row r="152" customFormat="1" s="486"/>
-    <row r="153" customFormat="1" s="486"/>
-    <row r="154" customFormat="1" s="486"/>
-    <row r="155" customFormat="1" s="486"/>
-    <row r="156" customFormat="1" s="486"/>
-    <row r="157" customFormat="1" s="486"/>
-    <row r="158" customFormat="1" s="486"/>
-    <row r="159" customFormat="1" s="486"/>
-    <row r="160" customFormat="1" s="486"/>
-    <row r="161" customFormat="1" s="486"/>
-    <row r="162" customFormat="1" s="486"/>
-    <row r="163" customFormat="1" s="486"/>
-    <row r="164" customFormat="1" s="486"/>
-    <row r="165" customFormat="1" s="486"/>
-    <row r="166" customFormat="1" s="486"/>
-    <row r="167" customFormat="1" s="486"/>
-    <row r="168" customFormat="1" s="486"/>
-    <row r="169" customFormat="1" s="486"/>
-    <row r="170" customFormat="1" s="486"/>
-    <row r="171" customFormat="1" s="486"/>
-    <row r="172" customFormat="1" s="486"/>
-    <row r="173" customFormat="1" s="486"/>
-    <row r="174" customFormat="1" s="486"/>
-    <row r="175" customFormat="1" s="486"/>
-    <row r="176" customFormat="1" s="486"/>
-    <row r="177" customFormat="1" s="486"/>
-    <row r="178" customFormat="1" s="486"/>
-  </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="B10:B20"/>
-    <mergeCell ref="B47:L48"/>
-    <mergeCell ref="B51:L52"/>
-    <mergeCell ref="F22:F23"/>
-    <mergeCell ref="B27:M29"/>
-    <mergeCell ref="B56:L57"/>
-    <mergeCell ref="M5:N5"/>
-    <mergeCell ref="B42:L43"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="D22:D23"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="FFFFC000"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AN43"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.33203125" defaultRowHeight="15.6"/>
-  <cols>
-    <col width="1.33203125" customWidth="1" style="590" min="1" max="1"/>
-    <col width="23.5546875" customWidth="1" style="590" min="2" max="2"/>
-    <col width="45.33203125" customWidth="1" style="590" min="3" max="3"/>
-    <col width="31.44140625" customWidth="1" style="590" min="4" max="4"/>
-    <col width="13.44140625" bestFit="1" customWidth="1" style="1593" min="5" max="5"/>
-    <col width="12.33203125" customWidth="1" style="1593" min="6" max="7"/>
-    <col width="10.33203125" customWidth="1" style="590" min="8" max="8"/>
-    <col width="12.33203125" customWidth="1" style="590" min="9" max="16384"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26.25" customFormat="1" customHeight="1" s="1593">
-      <c r="A1" s="590" t="n"/>
-      <c r="B1" s="1028" t="n"/>
-      <c r="H1" s="590" t="n"/>
-      <c r="I1" s="590" t="n"/>
-    </row>
-    <row r="2" ht="33" customFormat="1" customHeight="1" s="1593">
-      <c r="A2" s="590" t="n"/>
-      <c r="B2" s="592" t="inlineStr">
-        <is>
-          <t>LIQUIDADOR DE ANTICIPO DE RENTA</t>
-        </is>
-      </c>
-      <c r="C2" s="593" t="n"/>
-      <c r="D2" s="594" t="n"/>
-      <c r="H2" s="590" t="n"/>
-      <c r="I2" s="590" t="n"/>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="1506">
-      <c r="B3" s="595" t="inlineStr">
-        <is>
-          <t>Art. 807 del ET</t>
-        </is>
-      </c>
-      <c r="C3" s="595" t="n"/>
-      <c r="D3" s="595" t="n"/>
-    </row>
-    <row r="4">
-      <c r="B4" s="1024" t="inlineStr">
-        <is>
-          <t>OPCION 1 (Año actual)</t>
-        </is>
-      </c>
-      <c r="C4" s="1528" t="n"/>
-      <c r="D4" s="1594" t="n"/>
-      <c r="H4" s="597" t="n"/>
-      <c r="I4" s="597" t="n"/>
-      <c r="J4" s="597" t="n"/>
-    </row>
-    <row r="5">
-      <c r="B5" s="1020" t="inlineStr">
-        <is>
-          <t>Impuesto Neto de Renta del año gravable actual</t>
-        </is>
-      </c>
-      <c r="C5" s="1528" t="n"/>
-      <c r="D5" s="1595">
-        <f>+'Impuesto mínimo'!E36</f>
-        <v/>
-      </c>
-      <c r="H5" s="597" t="n"/>
-      <c r="I5" s="597" t="n"/>
-      <c r="J5" s="597" t="n"/>
-    </row>
-    <row r="6">
-      <c r="B6" s="1029" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="C6" s="1544" t="n"/>
-      <c r="D6" s="1596">
-        <f>ROUND(+D5*B6,-3)</f>
-        <v/>
-      </c>
-      <c r="H6" s="597" t="n"/>
-      <c r="I6" s="597" t="n"/>
-      <c r="J6" s="597" t="n"/>
-    </row>
-    <row r="7">
-      <c r="B7" s="1020" t="inlineStr">
-        <is>
-          <t>Menos: Retenciones en la fuente a favor</t>
-        </is>
-      </c>
-      <c r="C7" s="1528" t="n"/>
-      <c r="D7" s="1597">
-        <f>SUM('110'!AC48:AH48)</f>
-        <v/>
-      </c>
-      <c r="H7" s="597" t="n"/>
-      <c r="I7" s="597" t="n"/>
-      <c r="J7" s="597" t="n"/>
-    </row>
-    <row r="8">
-      <c r="B8" s="1021" t="inlineStr">
-        <is>
-          <t>ANTICIPO OPCION 1</t>
-        </is>
-      </c>
-      <c r="C8" s="1528" t="n"/>
-      <c r="D8" s="1598">
-        <f>IF(D6-D7&lt;0,0,D6-D7)</f>
-        <v/>
-      </c>
-      <c r="H8" s="597" t="n"/>
-      <c r="I8" s="597" t="n"/>
-      <c r="J8" s="597" t="n"/>
-    </row>
-    <row r="9" ht="13.5" customHeight="1" s="1506">
-      <c r="B9" s="602" t="n"/>
-      <c r="C9" s="602" t="n"/>
-      <c r="D9" s="1599" t="n"/>
-      <c r="H9" s="597" t="n"/>
-      <c r="I9" s="597" t="n"/>
-      <c r="J9" s="597" t="n"/>
-    </row>
-    <row r="10">
-      <c r="B10" s="1024" t="inlineStr">
-        <is>
-          <t>OPCION 2  (Promedio)</t>
-        </is>
-      </c>
-      <c r="C10" s="1528" t="n"/>
-      <c r="D10" s="1596" t="n"/>
-      <c r="H10" s="597" t="n"/>
-      <c r="I10" s="597" t="n"/>
-      <c r="J10" s="597" t="n"/>
-    </row>
-    <row r="11">
-      <c r="B11" s="1020" t="inlineStr">
-        <is>
-          <t>Impuesto Neto de Renta año anterior</t>
-        </is>
-      </c>
-      <c r="C11" s="1528" t="n"/>
-      <c r="D11" s="1597" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="1600">
-        <f>IF(AND(D12&gt;0,D11=0),"&lt;&lt; Digite el valor del impuesto neto de renta del año anterior","")</f>
-        <v/>
-      </c>
-      <c r="H11" s="597" t="n"/>
-      <c r="I11" s="597" t="n"/>
-      <c r="J11" s="597" t="n"/>
-    </row>
-    <row r="12">
-      <c r="B12" s="1020" t="inlineStr">
-        <is>
-          <t>Impuesto Neto de Renta del año gravable</t>
-        </is>
-      </c>
-      <c r="C12" s="1528" t="n"/>
-      <c r="D12" s="1597">
-        <f>+D5</f>
-        <v/>
-      </c>
-      <c r="H12" s="597" t="n"/>
-      <c r="I12" s="597" t="n"/>
-      <c r="J12" s="597" t="n"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="1025" t="inlineStr">
-        <is>
-          <t>Subtotal</t>
-        </is>
-      </c>
-      <c r="C13" s="1528" t="n"/>
-      <c r="D13" s="1601">
-        <f>+D11+D12</f>
-        <v/>
-      </c>
-      <c r="H13" s="597" t="n"/>
-      <c r="I13" s="597" t="n"/>
-      <c r="J13" s="597" t="n"/>
-    </row>
-    <row r="14">
-      <c r="B14" s="1026" t="inlineStr">
-        <is>
-          <t>Promedio</t>
-        </is>
-      </c>
-      <c r="C14" s="1528" t="n"/>
-      <c r="D14" s="1596">
-        <f>D13/2</f>
-        <v/>
-      </c>
-      <c r="H14" s="597" t="n"/>
-      <c r="I14" s="597" t="n"/>
-      <c r="J14" s="597" t="n"/>
-    </row>
-    <row r="15" customFormat="1" s="1593">
-      <c r="A15" s="590" t="n"/>
-      <c r="B15" s="1027">
-        <f>B6</f>
-        <v/>
-      </c>
-      <c r="C15" s="1528" t="n"/>
-      <c r="D15" s="1596">
-        <f>IF(B15&gt;25%,D14*B15,0)</f>
-        <v/>
-      </c>
-      <c r="H15" s="597" t="n"/>
-      <c r="I15" s="597" t="n"/>
-    </row>
-    <row r="16" customFormat="1" s="1593">
-      <c r="A16" s="590" t="n"/>
-      <c r="B16" s="1020" t="inlineStr">
-        <is>
-          <t>Menos: Retenciones en la fuente a favor</t>
-        </is>
-      </c>
-      <c r="C16" s="1528" t="n"/>
-      <c r="D16" s="1602">
-        <f>+D7</f>
-        <v/>
-      </c>
-      <c r="H16" s="597" t="n"/>
-      <c r="I16" s="597" t="n"/>
-    </row>
-    <row r="17" customFormat="1" s="1593">
-      <c r="A17" s="590" t="n"/>
-      <c r="B17" s="1021" t="inlineStr">
-        <is>
-          <t>ANTICIPO OPCION 2</t>
-        </is>
-      </c>
-      <c r="C17" s="1528" t="n"/>
-      <c r="D17" s="1598">
-        <f>IF(D15-D16&lt;0,0,D15-D16)</f>
-        <v/>
-      </c>
-      <c r="H17" s="597" t="n"/>
-      <c r="I17" s="597" t="n"/>
-    </row>
-    <row r="18" ht="3" customFormat="1" customHeight="1" s="1593">
-      <c r="A18" s="590" t="n"/>
-      <c r="B18" s="602" t="n"/>
-      <c r="C18" s="602" t="n"/>
-      <c r="D18" s="1599" t="n"/>
-      <c r="H18" s="597" t="n"/>
-      <c r="I18" s="597" t="n"/>
-    </row>
-    <row r="19" customFormat="1" s="1593">
-      <c r="A19" s="590" t="n"/>
-      <c r="B19" s="1022" t="inlineStr">
-        <is>
-          <t>VALOR DEL ANTICIPO AÑO SIGUIENTE</t>
-        </is>
-      </c>
-      <c r="C19" s="1528" t="n"/>
-      <c r="D19" s="1603">
-        <f>IF(B6=25%,D8,MIN(D8,D17))</f>
-        <v/>
-      </c>
-      <c r="H19" s="597" t="n"/>
-      <c r="I19" s="597" t="n"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="597" t="n"/>
-      <c r="C20" s="597" t="n"/>
-      <c r="D20" s="597" t="n"/>
-      <c r="H20" s="597" t="n"/>
-      <c r="I20" s="597" t="n"/>
-      <c r="J20" s="597" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="597" t="inlineStr"/>
-      <c r="C21" s="597" t="n"/>
-      <c r="D21" s="597" t="n"/>
-      <c r="H21" s="597" t="n"/>
-      <c r="I21" s="597" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="597" t="n"/>
-      <c r="C22" s="597" t="n"/>
-      <c r="D22" s="597" t="n"/>
-      <c r="H22" s="597" t="n"/>
-      <c r="I22" s="597" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="597" t="n"/>
-      <c r="C23" s="597" t="n"/>
-      <c r="D23" s="597" t="n"/>
-      <c r="H23" s="597" t="n"/>
-      <c r="I23" s="597" t="n"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="597" t="n"/>
-      <c r="C24" s="597" t="n"/>
-      <c r="D24" s="597" t="n"/>
-      <c r="H24" s="597" t="n"/>
-      <c r="I24" s="597" t="n"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="597" t="n"/>
-      <c r="C25" s="597" t="n"/>
-      <c r="D25" s="597" t="n"/>
-      <c r="H25" s="597" t="n"/>
-      <c r="I25" s="597" t="n"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="597" t="n"/>
-      <c r="C26" s="597" t="n"/>
-      <c r="D26" s="597" t="n"/>
-      <c r="H26" s="597" t="n"/>
-      <c r="I26" s="597" t="n"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="597" t="n"/>
-      <c r="C27" s="597" t="n"/>
-      <c r="D27" s="597" t="n"/>
-      <c r="H27" s="597" t="n"/>
-      <c r="I27" s="597" t="n"/>
-    </row>
-    <row r="28">
-      <c r="B28" s="597" t="n"/>
-      <c r="C28" s="597" t="n"/>
-      <c r="D28" s="597" t="n"/>
-      <c r="H28" s="597" t="n"/>
-      <c r="I28" s="597" t="n"/>
-    </row>
-    <row r="29">
-      <c r="B29" s="597" t="n"/>
-      <c r="C29" s="597" t="n"/>
-      <c r="D29" s="597" t="n"/>
-      <c r="H29" s="597" t="n"/>
-      <c r="I29" s="597" t="n"/>
-    </row>
-    <row r="30">
-      <c r="B30" s="597" t="n"/>
-      <c r="C30" s="597" t="n"/>
-      <c r="D30" s="597" t="n"/>
-      <c r="H30" s="597" t="n"/>
-      <c r="I30" s="597" t="n"/>
-    </row>
-    <row r="31">
-      <c r="B31" s="597" t="n"/>
-      <c r="C31" s="597" t="n"/>
-      <c r="D31" s="597" t="n"/>
-      <c r="H31" s="597" t="n"/>
-      <c r="I31" s="597" t="n"/>
-    </row>
-    <row r="32">
-      <c r="B32" s="597" t="n"/>
-      <c r="C32" s="597" t="n"/>
-      <c r="D32" s="597" t="n"/>
-      <c r="H32" s="597" t="n"/>
-      <c r="I32" s="597" t="n"/>
-    </row>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39">
-      <c r="B39" s="608" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="608" t="n">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="608" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="B42" s="608" t="n">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" s="608" t="n"/>
-    </row>
-  </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" algorithmName="SHA-512" sheet="1" objects="1" insertRows="1" insertHyperlinks="0" autoFilter="0" scenarios="1" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" saltValue="d8/754m7aeojz5pxqbD7Jg==" formatRows="0" sort="0" spinCount="100000" hashValue="x6C4DFWiHgnnNLk2A93OOFpqn3c3G5kRySEsPovsseJno221alpsJb53RUfMl971RgvyOFx+m19/O7BTlULtZQ=="/>
-  <mergeCells count="15">
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B12:C12"/>
-  </mergeCells>
-  <dataValidations disablePrompts="1" count="2">
-    <dataValidation sqref="D7" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" prompt="Incluya las retenciones en la fuente a favor, y tambien las autorretenciones si considera que se pueden restar."/>
-    <dataValidation sqref="B6:C6" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" prompt="Seleccione de la lista o digite 0%, 25%, 50%, o 75% según corresponda" type="list">
-      <formula1>$B$39:$B$42</formula1>
-    </dataValidation>
-  </dataValidations>
-  <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.3149606299212598" right="0.3149606299212598" top="0.5511811023622047" bottom="0.3543307086614174" header="0.3149606299212598" footer="0.3149606299212598"/>
-  <pageSetup orientation="portrait" scale="90" horizontalDpi="0" verticalDpi="0"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;L&amp;D&amp;T&amp;Cwww.consultorcontable.com&amp;RLiquidador de anticipo de renta</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-</worksheet>
 </file>
</xml_diff>